<commit_message>
Added assistance data to tables and added two assistance scripts to script list in initialized database
</commit_message>
<xml_diff>
--- a/assistance/assistance_programs.xlsx
+++ b/assistance/assistance_programs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nataliealba/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nataliealba/Desktop/untitled folder/CS_316_Project/assistance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55597C5C-4D7C-214B-AEE6-D4EEC8C51983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E76B44CA-9ED4-7643-99AD-44C280D6F9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="311">
   <si>
     <t>program_id</t>
   </si>
@@ -953,6 +953,9 @@
   </si>
   <si>
     <t>All 30 original Coding Ready program IDs preserved, including omission of P008.</t>
+  </si>
+  <si>
+    <t>P008</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1285,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="3" width="30" customWidth="1"/>
@@ -2793,7 +2796,7 @@
     </row>
     <row r="31" spans="1:19" ht="66" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>259</v>
+        <v>310</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>260</v>
@@ -2845,7 +2848,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="39" customWidth="1"/>
@@ -4175,7 +4178,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
@@ -4301,7 +4304,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="16">
+    <row r="16" spans="1:2" ht="15">
       <c r="A16" s="1" t="s">
         <v>306</v>
       </c>
@@ -4309,7 +4312,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="16">
+    <row r="17" spans="1:2" ht="15">
       <c r="A17" s="1" t="s">
         <v>308</v>
       </c>

</xml_diff>